<commit_message>
#70 Control Board BOM Updated
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/Control_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/Control_BOM-Control-Board.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0C6FF5-C51C-4D46-A49B-A28E1647E86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -718,7 +719,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1157,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1263,12 +1264,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1691,7 +1686,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1714,8 +1709,8 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="64"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="62"/>
     </row>
     <row r="2" spans="1:10" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1730,8 +1725,8 @@
       <c r="F2" s="11"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="72"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="70"/>
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1747,7 +1742,7 @@
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="65"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1763,7 +1758,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
-      <c r="J4" s="66"/>
+      <c r="J4" s="64"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1779,7 +1774,7 @@
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
-      <c r="J5" s="66"/>
+      <c r="J5" s="64"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1791,7 +1786,7 @@
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
-      <c r="J6" s="66"/>
+      <c r="J6" s="64"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1803,491 +1798,494 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
-      <c r="J7" s="66"/>
+      <c r="J7" s="64"/>
     </row>
     <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="41"/>
       <c r="C8" s="37"/>
       <c r="D8" s="37"/>
-      <c r="E8" s="44"/>
+      <c r="E8" s="42"/>
       <c r="F8" s="17"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="66"/>
+      <c r="J8" s="64"/>
     </row>
     <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="50" t="s">
+      <c r="D9" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="48" t="s">
+      <c r="E9" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="F9" s="50" t="s">
+      <c r="F9" s="48" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="48" t="s">
+      <c r="G9" s="46" t="s">
         <v>148</v>
       </c>
-      <c r="H9" s="50" t="s">
+      <c r="H9" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="I9" s="48" t="s">
+      <c r="I9" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="J9" s="49" t="s">
+      <c r="J9" s="47" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="45">
+      <c r="B10" s="43">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="51" t="s">
+      <c r="D10" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="46" t="s">
+      <c r="E10" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="51" t="s">
+      <c r="F10" s="49" t="s">
         <v>122</v>
       </c>
-      <c r="G10" s="46" t="s">
+      <c r="G10" s="44" t="s">
         <v>149</v>
       </c>
-      <c r="H10" s="51" t="s">
+      <c r="H10" s="49" t="s">
         <v>175</v>
       </c>
-      <c r="I10" s="58">
+      <c r="I10" s="56">
         <v>3</v>
       </c>
-      <c r="J10" s="47">
+      <c r="J10" s="45">
         <f>I10*5</f>
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="42">
+      <c r="B11" s="43">
         <f t="shared" ref="B11:B54" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="39" t="s">
         <v>217</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="50" t="s">
         <v>51</v>
       </c>
       <c r="E11" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="F11" s="52" t="s">
+      <c r="F11" s="50" t="s">
         <v>123</v>
       </c>
       <c r="G11" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="H11" s="52" t="s">
+      <c r="H11" s="50" t="s">
         <v>176</v>
       </c>
-      <c r="I11" s="59">
+      <c r="I11" s="57">
         <v>24</v>
       </c>
-      <c r="J11" s="62">
+      <c r="J11" s="60">
         <f t="shared" ref="J11:J54" si="1">I11*5</f>
         <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="42">
-        <f>ROW(B12) - ROW($B$9)</f>
+      <c r="B12" s="43">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C12" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="53" t="s">
+      <c r="D12" s="51" t="s">
         <v>52</v>
       </c>
       <c r="E12" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="F12" s="53" t="s">
+      <c r="F12" s="51" t="s">
         <v>124</v>
       </c>
       <c r="G12" s="38" t="s">
         <v>150</v>
       </c>
-      <c r="H12" s="53" t="s">
+      <c r="H12" s="51" t="s">
         <v>177</v>
       </c>
-      <c r="I12" s="60">
+      <c r="I12" s="58">
         <v>1</v>
       </c>
-      <c r="J12" s="47">
+      <c r="J12" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="42">
+      <c r="B13" s="43">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="52" t="s">
+      <c r="D13" s="50" t="s">
         <v>53</v>
       </c>
       <c r="E13" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="F13" s="52" t="s">
+      <c r="F13" s="50" t="s">
         <v>125</v>
       </c>
       <c r="G13" s="39" t="s">
         <v>151</v>
       </c>
-      <c r="H13" s="52" t="s">
+      <c r="H13" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="I13" s="59">
+      <c r="I13" s="57">
         <v>8</v>
       </c>
-      <c r="J13" s="62">
+      <c r="J13" s="60">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="42">
-        <f>ROW(B14) - ROW($B$9)</f>
+      <c r="B14" s="43">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C14" s="38" t="s">
         <v>218</v>
       </c>
-      <c r="D14" s="53" t="s">
+      <c r="D14" s="51" t="s">
         <v>54</v>
       </c>
       <c r="E14" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="F14" s="53" t="s">
+      <c r="F14" s="51" t="s">
         <v>126</v>
       </c>
       <c r="G14" s="38" t="s">
         <v>152</v>
       </c>
-      <c r="H14" s="53" t="s">
+      <c r="H14" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="I14" s="60">
+      <c r="I14" s="58">
         <v>2</v>
       </c>
-      <c r="J14" s="47">
+      <c r="J14" s="45">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="42">
+      <c r="B15" s="43">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="39" t="s">
         <v>219</v>
       </c>
-      <c r="D15" s="52" t="s">
+      <c r="D15" s="50" t="s">
         <v>55</v>
       </c>
       <c r="E15" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="F15" s="52" t="s">
+      <c r="F15" s="50" t="s">
         <v>127</v>
       </c>
       <c r="G15" s="39" t="s">
         <v>151</v>
       </c>
-      <c r="H15" s="52" t="s">
+      <c r="H15" s="50" t="s">
         <v>180</v>
       </c>
-      <c r="I15" s="59">
+      <c r="I15" s="57">
         <v>7</v>
       </c>
-      <c r="J15" s="62">
+      <c r="J15" s="60">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="42">
-        <f>ROW(B16) - ROW($B$9)</f>
+      <c r="B16" s="43">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C16" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="53" t="s">
+      <c r="D16" s="51" t="s">
         <v>56</v>
       </c>
       <c r="E16" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="F16" s="53" t="s">
+      <c r="F16" s="51" t="s">
         <v>128</v>
       </c>
       <c r="G16" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="H16" s="53" t="s">
+      <c r="H16" s="51" t="s">
         <v>181</v>
       </c>
-      <c r="I16" s="60">
+      <c r="I16" s="58">
         <v>1</v>
       </c>
-      <c r="J16" s="47">
+      <c r="J16" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="42"/>
+      <c r="B17" s="43">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
       <c r="C17" s="38" t="s">
         <v>220</v>
       </c>
-      <c r="D17" s="53" t="s">
+      <c r="D17" s="51" t="s">
         <v>223</v>
       </c>
       <c r="E17" s="38" t="s">
         <v>221</v>
       </c>
-      <c r="F17" s="53" t="s">
+      <c r="F17" s="51" t="s">
         <v>222</v>
       </c>
       <c r="G17" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="H17" s="53" t="s">
+      <c r="H17" s="51" t="s">
         <v>224</v>
       </c>
-      <c r="I17" s="60">
+      <c r="I17" s="58">
         <v>1</v>
       </c>
-      <c r="J17" s="47">
+      <c r="J17" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="42">
+      <c r="B18" s="43">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="D18" s="52" t="s">
+      <c r="D18" s="50" t="s">
         <v>204</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="52" t="s">
+      <c r="F18" s="50" t="s">
         <v>203</v>
       </c>
       <c r="G18" s="39" t="s">
         <v>151</v>
       </c>
-      <c r="H18" s="52" t="s">
+      <c r="H18" s="50" t="s">
         <v>182</v>
       </c>
-      <c r="I18" s="59">
-        <v>2</v>
-      </c>
-      <c r="J18" s="62">
-        <f t="shared" si="1"/>
-        <v>10</v>
+      <c r="I18" s="57">
+        <v>1</v>
+      </c>
+      <c r="J18" s="60">
+        <f t="shared" si="1"/>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="42">
-        <f>ROW(B19) - ROW($B$9)</f>
+      <c r="B19" s="43">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="53" t="s">
+      <c r="D19" s="51" t="s">
         <v>57</v>
       </c>
       <c r="E19" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="F19" s="53" t="s">
+      <c r="F19" s="51" t="s">
         <v>129</v>
       </c>
       <c r="G19" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="H19" s="53" t="s">
+      <c r="H19" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="I19" s="60">
+      <c r="I19" s="58">
         <v>1</v>
       </c>
-      <c r="J19" s="47">
+      <c r="J19" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="42">
+      <c r="B20" s="43">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="52" t="s">
+      <c r="D20" s="50" t="s">
         <v>58</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="F20" s="52" t="s">
+      <c r="F20" s="50" t="s">
         <v>93</v>
       </c>
       <c r="G20" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="H20" s="55" t="s">
+      <c r="H20" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="I20" s="59">
+      <c r="I20" s="57">
         <v>1</v>
       </c>
-      <c r="J20" s="62">
+      <c r="J20" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="42">
-        <f>ROW(B21) - ROW($B$9)</f>
+      <c r="B21" s="43">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C21" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="51" t="s">
         <v>59</v>
       </c>
       <c r="E21" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F21" s="53" t="s">
+      <c r="F21" s="51" t="s">
         <v>94</v>
       </c>
       <c r="G21" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="H21" s="57" t="s">
+      <c r="H21" s="55" t="s">
         <v>201</v>
       </c>
-      <c r="I21" s="60">
+      <c r="I21" s="58">
         <v>1</v>
       </c>
-      <c r="J21" s="47">
+      <c r="J21" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="42">
+      <c r="B22" s="43">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C22" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="52" t="s">
+      <c r="D22" s="50" t="s">
         <v>60</v>
       </c>
       <c r="E22" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="F22" s="52" t="s">
+      <c r="F22" s="50" t="s">
         <v>95</v>
       </c>
       <c r="G22" s="39" t="s">
         <v>155</v>
       </c>
-      <c r="H22" s="55" t="s">
+      <c r="H22" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="I22" s="59">
+      <c r="I22" s="57">
         <v>1</v>
       </c>
-      <c r="J22" s="62">
+      <c r="J22" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="42">
-        <f>ROW(B23) - ROW($B$9)</f>
+      <c r="B23" s="43">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="51" t="s">
         <v>61</v>
       </c>
       <c r="E23" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F23" s="53" t="s">
+      <c r="F23" s="51" t="s">
         <v>96</v>
       </c>
       <c r="G23" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="H23" s="57" t="s">
+      <c r="H23" s="55" t="s">
         <v>201</v>
       </c>
-      <c r="I23" s="60">
+      <c r="I23" s="58">
         <v>1</v>
       </c>
-      <c r="J23" s="47">
+      <c r="J23" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -2301,352 +2299,352 @@
       <c r="C24" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="D24" s="52" t="s">
+      <c r="D24" s="50" t="s">
         <v>205</v>
       </c>
       <c r="E24" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="F24" s="52" t="s">
+      <c r="F24" s="50" t="s">
         <v>206</v>
       </c>
-      <c r="G24" s="56" t="s">
+      <c r="G24" s="54" t="s">
         <v>207</v>
       </c>
-      <c r="H24" s="55" t="s">
+      <c r="H24" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="I24" s="59">
+      <c r="I24" s="57">
         <v>1</v>
       </c>
-      <c r="J24" s="62">
+      <c r="J24" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="42">
-        <f>ROW(B25) - ROW($B$9)</f>
+      <c r="B25" s="43">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="D25" s="53" t="s">
+      <c r="D25" s="51" t="s">
         <v>62</v>
       </c>
       <c r="E25" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F25" s="53" t="s">
+      <c r="F25" s="51" t="s">
         <v>98</v>
       </c>
       <c r="G25" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="H25" s="57" t="s">
+      <c r="H25" s="55" t="s">
         <v>201</v>
       </c>
-      <c r="I25" s="60">
+      <c r="I25" s="58">
         <v>1</v>
       </c>
-      <c r="J25" s="47">
+      <c r="J25" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="42">
+      <c r="B26" s="43">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="D26" s="52" t="s">
+      <c r="D26" s="50" t="s">
         <v>208</v>
       </c>
       <c r="E26" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="F26" s="52" t="s">
+      <c r="F26" s="50" t="s">
         <v>209</v>
       </c>
-      <c r="G26" s="56" t="s">
+      <c r="G26" s="54" t="s">
         <v>207</v>
       </c>
-      <c r="H26" s="55" t="s">
+      <c r="H26" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="I26" s="59">
+      <c r="I26" s="57">
         <v>1</v>
       </c>
-      <c r="J26" s="62">
+      <c r="J26" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="42">
-        <f>ROW(B27) - ROW($B$9)</f>
+      <c r="B27" s="43">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C27" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="D27" s="53" t="s">
+      <c r="D27" s="51" t="s">
         <v>63</v>
       </c>
       <c r="E27" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F27" s="53" t="s">
+      <c r="F27" s="51" t="s">
         <v>100</v>
       </c>
       <c r="G27" s="38" t="s">
         <v>152</v>
       </c>
-      <c r="H27" s="53" t="s">
+      <c r="H27" s="51" t="s">
         <v>184</v>
       </c>
-      <c r="I27" s="60">
+      <c r="I27" s="58">
         <v>1</v>
       </c>
-      <c r="J27" s="47">
+      <c r="J27" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="42">
-        <f>ROW(B28) - ROW($B$9)</f>
+      <c r="B28" s="43">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C28" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="53" t="s">
+      <c r="D28" s="51" t="s">
         <v>64</v>
       </c>
       <c r="E28" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="F28" s="53" t="s">
+      <c r="F28" s="51" t="s">
         <v>130</v>
       </c>
       <c r="G28" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="H28" s="53" t="s">
+      <c r="H28" s="51" t="s">
         <v>185</v>
       </c>
-      <c r="I28" s="60">
+      <c r="I28" s="58">
         <v>1</v>
       </c>
-      <c r="J28" s="47">
+      <c r="J28" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="42">
+      <c r="B29" s="43">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C29" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D29" s="52" t="s">
+      <c r="D29" s="50" t="s">
         <v>65</v>
       </c>
       <c r="E29" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="F29" s="52" t="s">
+      <c r="F29" s="50" t="s">
         <v>102</v>
       </c>
       <c r="G29" s="39" t="s">
         <v>158</v>
       </c>
-      <c r="H29" s="52" t="s">
+      <c r="H29" s="50" t="s">
         <v>186</v>
       </c>
-      <c r="I29" s="59">
+      <c r="I29" s="57">
         <v>1</v>
       </c>
-      <c r="J29" s="62">
+      <c r="J29" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="42">
-        <f>ROW(B30) - ROW($B$9)</f>
+      <c r="B30" s="43">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C30" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="53" t="s">
+      <c r="D30" s="51" t="s">
         <v>66</v>
       </c>
       <c r="E30" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="F30" s="53" t="s">
+      <c r="F30" s="51" t="s">
         <v>131</v>
       </c>
       <c r="G30" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="H30" s="53" t="s">
+      <c r="H30" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="I30" s="60">
+      <c r="I30" s="58">
         <v>1</v>
       </c>
-      <c r="J30" s="47">
+      <c r="J30" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="B31" s="42">
+      <c r="B31" s="43">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C31" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="D31" s="52" t="s">
+      <c r="D31" s="50" t="s">
         <v>67</v>
       </c>
       <c r="E31" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="F31" s="52" t="s">
+      <c r="F31" s="50" t="s">
         <v>132</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="H31" s="55" t="s">
+      <c r="H31" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I31" s="59">
+      <c r="I31" s="57">
         <v>1</v>
       </c>
-      <c r="J31" s="62">
+      <c r="J31" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="42">
-        <f>ROW(B32) - ROW($B$9)</f>
+      <c r="B32" s="43">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C32" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="53" t="s">
+      <c r="D32" s="51" t="s">
         <v>68</v>
       </c>
       <c r="E32" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F32" s="53" t="s">
+      <c r="F32" s="51" t="s">
         <v>104</v>
       </c>
       <c r="G32" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="H32" s="53" t="s">
+      <c r="H32" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="I32" s="60">
+      <c r="I32" s="58">
         <v>1</v>
       </c>
-      <c r="J32" s="47">
+      <c r="J32" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="42">
+      <c r="B33" s="43">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C33" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="D33" s="52" t="s">
+      <c r="D33" s="50" t="s">
         <v>69</v>
       </c>
       <c r="E33" s="39" t="s">
         <v>105</v>
       </c>
-      <c r="F33" s="52" t="s">
+      <c r="F33" s="50" t="s">
         <v>133</v>
       </c>
       <c r="G33" s="39" t="s">
         <v>160</v>
       </c>
-      <c r="H33" s="55" t="s">
+      <c r="H33" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I33" s="59">
+      <c r="I33" s="57">
         <v>2</v>
       </c>
-      <c r="J33" s="62">
+      <c r="J33" s="60">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="42">
-        <f>ROW(B34) - ROW($B$9)</f>
+      <c r="B34" s="43">
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C34" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="D34" s="53" t="s">
+      <c r="D34" s="51" t="s">
         <v>70</v>
       </c>
       <c r="E34" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="F34" s="53" t="s">
+      <c r="F34" s="51" t="s">
         <v>134</v>
       </c>
       <c r="G34" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="H34" s="57" t="s">
+      <c r="H34" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="I34" s="60">
+      <c r="I34" s="58">
         <v>1</v>
       </c>
-      <c r="J34" s="47">
+      <c r="J34" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
-      <c r="B35" s="42">
+      <c r="B35" s="43">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
@@ -2659,27 +2657,27 @@
       <c r="E35" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="F35" s="52" t="s">
+      <c r="F35" s="50" t="s">
         <v>211</v>
       </c>
       <c r="G35" s="39" t="s">
         <v>212</v>
       </c>
-      <c r="H35" s="52" t="s">
+      <c r="H35" s="50" t="s">
         <v>189</v>
       </c>
-      <c r="I35" s="59">
+      <c r="I35" s="57">
         <v>1</v>
       </c>
-      <c r="J35" s="62">
+      <c r="J35" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="42">
-        <f>ROW(B36) - ROW($B$9)</f>
+      <c r="B36" s="43">
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C36" s="38" t="s">
@@ -2697,589 +2695,589 @@
       <c r="G36" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="H36" s="53" t="s">
+      <c r="H36" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="I36" s="60">
+      <c r="I36" s="58">
         <v>4</v>
       </c>
-      <c r="J36" s="47">
+      <c r="J36" s="45">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
-      <c r="B37" s="42">
+      <c r="B37" s="43">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C37" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="D37" s="52" t="s">
+      <c r="D37" s="50" t="s">
         <v>71</v>
       </c>
       <c r="E37" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="F37" s="52" t="s">
+      <c r="F37" s="50" t="s">
         <v>135</v>
       </c>
       <c r="G37" s="39" t="s">
         <v>151</v>
       </c>
-      <c r="H37" s="52" t="s">
+      <c r="H37" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="I37" s="59">
+      <c r="I37" s="57">
         <v>10</v>
       </c>
-      <c r="J37" s="62">
+      <c r="J37" s="60">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="42">
+      <c r="B38" s="43">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C38" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="D38" s="52" t="s">
+      <c r="D38" s="50" t="s">
         <v>72</v>
       </c>
       <c r="E38" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="F38" s="52" t="s">
+      <c r="F38" s="50" t="s">
         <v>136</v>
       </c>
       <c r="G38" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="H38" s="52" t="s">
+      <c r="H38" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="I38" s="59">
+      <c r="I38" s="57">
         <v>8</v>
       </c>
-      <c r="J38" s="62">
+      <c r="J38" s="60">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="42">
-        <f>ROW(B39) - ROW($B$9)</f>
+      <c r="B39" s="43">
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="D39" s="53" t="s">
+      <c r="D39" s="51" t="s">
         <v>73</v>
       </c>
       <c r="E39" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="F39" s="53" t="s">
+      <c r="F39" s="51" t="s">
         <v>137</v>
       </c>
       <c r="G39" s="38" t="s">
         <v>161</v>
       </c>
-      <c r="H39" s="53" t="s">
+      <c r="H39" s="51" t="s">
         <v>193</v>
       </c>
-      <c r="I39" s="60">
+      <c r="I39" s="58">
         <v>2</v>
       </c>
-      <c r="J39" s="47">
+      <c r="J39" s="45">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="42">
+      <c r="B40" s="43">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C40" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="52" t="s">
+      <c r="D40" s="50" t="s">
         <v>74</v>
       </c>
       <c r="E40" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="F40" s="52" t="s">
+      <c r="F40" s="50" t="s">
         <v>138</v>
       </c>
       <c r="G40" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="H40" s="52" t="s">
+      <c r="H40" s="50" t="s">
         <v>194</v>
       </c>
-      <c r="I40" s="59">
+      <c r="I40" s="57">
         <v>2</v>
       </c>
-      <c r="J40" s="62">
+      <c r="J40" s="60">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="42">
-        <f>ROW(B41) - ROW($B$9)</f>
+      <c r="B41" s="43">
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="D41" s="53" t="s">
+      <c r="D41" s="51" t="s">
         <v>75</v>
       </c>
       <c r="E41" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="F41" s="53" t="s">
+      <c r="F41" s="51" t="s">
         <v>139</v>
       </c>
       <c r="G41" s="38" t="s">
         <v>151</v>
       </c>
-      <c r="H41" s="53" t="s">
+      <c r="H41" s="51" t="s">
         <v>195</v>
       </c>
-      <c r="I41" s="60">
+      <c r="I41" s="58">
         <v>1</v>
       </c>
-      <c r="J41" s="47">
+      <c r="J41" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="42">
+      <c r="B42" s="43">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C42" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="D42" s="52" t="s">
+      <c r="D42" s="50" t="s">
         <v>76</v>
       </c>
       <c r="E42" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="F42" s="55" t="s">
+      <c r="F42" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="G42" s="56" t="s">
+      <c r="G42" s="54" t="s">
         <v>202</v>
       </c>
-      <c r="H42" s="55" t="s">
+      <c r="H42" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I42" s="59">
+      <c r="I42" s="57">
         <v>3</v>
       </c>
-      <c r="J42" s="62">
+      <c r="J42" s="60">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="42">
-        <f>ROW(B43) - ROW($B$9)</f>
+      <c r="B43" s="43">
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C43" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="D43" s="53" t="s">
+      <c r="D43" s="51" t="s">
         <v>77</v>
       </c>
       <c r="E43" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F43" s="53" t="s">
+      <c r="F43" s="51" t="s">
         <v>109</v>
       </c>
       <c r="G43" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="H43" s="57" t="s">
+      <c r="H43" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="I43" s="60">
+      <c r="I43" s="58">
         <v>2</v>
       </c>
-      <c r="J43" s="47">
+      <c r="J43" s="45">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
-      <c r="B44" s="42">
+      <c r="B44" s="43">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C44" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="D44" s="52" t="s">
+      <c r="D44" s="50" t="s">
         <v>78</v>
       </c>
       <c r="E44" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="F44" s="52" t="s">
+      <c r="F44" s="50" t="s">
         <v>140</v>
       </c>
       <c r="G44" s="39" t="s">
         <v>164</v>
       </c>
-      <c r="H44" s="55" t="s">
+      <c r="H44" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I44" s="59">
+      <c r="I44" s="57">
         <v>1</v>
       </c>
-      <c r="J44" s="62">
+      <c r="J44" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
-      <c r="B45" s="42">
-        <f>ROW(B45) - ROW($B$9)</f>
+      <c r="B45" s="43">
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C45" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="D45" s="53" t="s">
+      <c r="D45" s="51" t="s">
         <v>79</v>
       </c>
       <c r="E45" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="F45" s="53" t="s">
+      <c r="F45" s="51" t="s">
         <v>141</v>
       </c>
       <c r="G45" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="H45" s="57" t="s">
+      <c r="H45" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="I45" s="60">
+      <c r="I45" s="58">
         <v>1</v>
       </c>
-      <c r="J45" s="47">
+      <c r="J45" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
-      <c r="B46" s="42">
+      <c r="B46" s="43">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C46" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="D46" s="52" t="s">
+      <c r="D46" s="50" t="s">
         <v>80</v>
       </c>
       <c r="E46" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="F46" s="52" t="s">
+      <c r="F46" s="50" t="s">
         <v>142</v>
       </c>
       <c r="G46" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="H46" s="55" t="s">
+      <c r="H46" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I46" s="59">
+      <c r="I46" s="57">
         <v>1</v>
       </c>
-      <c r="J46" s="62">
+      <c r="J46" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
-      <c r="B47" s="42">
-        <f>ROW(B47) - ROW($B$9)</f>
+      <c r="B47" s="43">
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C47" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="D47" s="53" t="s">
+      <c r="D47" s="51" t="s">
         <v>81</v>
       </c>
       <c r="E47" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="F47" s="53" t="s">
+      <c r="F47" s="51" t="s">
         <v>143</v>
       </c>
       <c r="G47" s="38" t="s">
         <v>167</v>
       </c>
-      <c r="H47" s="57" t="s">
+      <c r="H47" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="I47" s="60">
+      <c r="I47" s="58">
         <v>1</v>
       </c>
-      <c r="J47" s="47">
+      <c r="J47" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
-      <c r="B48" s="42">
+      <c r="B48" s="43">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C48" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="D48" s="52" t="s">
+      <c r="D48" s="50" t="s">
         <v>82</v>
       </c>
       <c r="E48" s="39" t="s">
         <v>114</v>
       </c>
-      <c r="F48" s="52" t="s">
+      <c r="F48" s="50" t="s">
         <v>144</v>
       </c>
       <c r="G48" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="H48" s="55" t="s">
+      <c r="H48" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I48" s="59">
+      <c r="I48" s="57">
         <v>1</v>
       </c>
-      <c r="J48" s="62">
+      <c r="J48" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
-      <c r="B49" s="42">
-        <f>ROW(B49) - ROW($B$9)</f>
+      <c r="B49" s="43">
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C49" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="D49" s="53" t="s">
+      <c r="D49" s="51" t="s">
         <v>83</v>
       </c>
       <c r="E49" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="F49" s="53" t="s">
+      <c r="F49" s="51" t="s">
         <v>145</v>
       </c>
       <c r="G49" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="H49" s="57" t="s">
+      <c r="H49" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="I49" s="60">
+      <c r="I49" s="58">
         <v>1</v>
       </c>
-      <c r="J49" s="47">
+      <c r="J49" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
-      <c r="B50" s="42">
+      <c r="B50" s="43">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C50" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="D50" s="52" t="s">
+      <c r="D50" s="50" t="s">
         <v>84</v>
       </c>
       <c r="E50" s="39" t="s">
         <v>116</v>
       </c>
-      <c r="F50" s="52" t="s">
+      <c r="F50" s="50" t="s">
         <v>146</v>
       </c>
       <c r="G50" s="39" t="s">
         <v>170</v>
       </c>
-      <c r="H50" s="55" t="s">
+      <c r="H50" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="I50" s="59">
+      <c r="I50" s="57">
         <v>1</v>
       </c>
-      <c r="J50" s="62">
+      <c r="J50" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
-      <c r="B51" s="42">
-        <f>ROW(B51) - ROW($B$9)</f>
+      <c r="B51" s="43">
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="C51" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="D51" s="53" t="s">
+      <c r="D51" s="51" t="s">
         <v>85</v>
       </c>
       <c r="E51" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="F51" s="53" t="s">
+      <c r="F51" s="51" t="s">
         <v>147</v>
       </c>
       <c r="G51" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="H51" s="57" t="s">
+      <c r="H51" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="I51" s="60">
+      <c r="I51" s="58">
         <v>1</v>
       </c>
-      <c r="J51" s="47">
+      <c r="J51" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
-      <c r="B52" s="42">
+      <c r="B52" s="43">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="C52" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="D52" s="52" t="s">
+      <c r="D52" s="50" t="s">
         <v>86</v>
       </c>
       <c r="E52" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="F52" s="52" t="s">
+      <c r="F52" s="50" t="s">
         <v>118</v>
       </c>
       <c r="G52" s="39" t="s">
         <v>172</v>
       </c>
-      <c r="H52" s="52" t="s">
+      <c r="H52" s="50" t="s">
         <v>196</v>
       </c>
-      <c r="I52" s="59">
+      <c r="I52" s="57">
         <v>2</v>
       </c>
-      <c r="J52" s="62">
+      <c r="J52" s="60">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
-      <c r="B53" s="42">
-        <f>ROW(B53) - ROW($B$9)</f>
+      <c r="B53" s="43">
+        <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C53" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="D53" s="53" t="s">
+      <c r="D53" s="51" t="s">
         <v>87</v>
       </c>
       <c r="E53" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="F53" s="53" t="s">
+      <c r="F53" s="51" t="s">
         <v>119</v>
       </c>
       <c r="G53" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="H53" s="53" t="s">
+      <c r="H53" s="51" t="s">
         <v>197</v>
       </c>
-      <c r="I53" s="60">
+      <c r="I53" s="58">
         <v>1</v>
       </c>
-      <c r="J53" s="47">
+      <c r="J53" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="42">
+      <c r="B54" s="43">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="C54" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="D54" s="54" t="s">
+      <c r="D54" s="52" t="s">
         <v>88</v>
       </c>
       <c r="E54" s="40" t="s">
         <v>200</v>
       </c>
-      <c r="F54" s="54" t="s">
+      <c r="F54" s="52" t="s">
         <v>120</v>
       </c>
       <c r="G54" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="H54" s="54" t="s">
+      <c r="H54" s="52" t="s">
         <v>198</v>
       </c>
-      <c r="I54" s="61">
+      <c r="I54" s="59">
         <v>1</v>
       </c>
-      <c r="J54" s="62">
+      <c r="J54" s="60">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -3292,11 +3290,11 @@
       </c>
       <c r="D55" s="35"/>
       <c r="E55" s="36"/>
-      <c r="F55" s="67"/>
-      <c r="G55" s="67"/>
-      <c r="H55" s="67"/>
-      <c r="I55" s="67"/>
-      <c r="J55" s="68"/>
+      <c r="F55" s="65"/>
+      <c r="G55" s="65"/>
+      <c r="H55" s="65"/>
+      <c r="I55" s="65"/>
+      <c r="J55" s="66"/>
     </row>
     <row r="56" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
@@ -3306,11 +3304,11 @@
       </c>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
-      <c r="F56" s="69"/>
-      <c r="G56" s="69"/>
-      <c r="H56" s="69"/>
-      <c r="I56" s="69"/>
-      <c r="J56" s="70"/>
+      <c r="F56" s="67"/>
+      <c r="G56" s="67"/>
+      <c r="H56" s="67"/>
+      <c r="I56" s="67"/>
+      <c r="J56" s="68"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>